<commit_message>
gitignore update and som else
</commit_message>
<xml_diff>
--- a/pandas/to_excel.xlsx
+++ b/pandas/to_excel.xlsx
@@ -3,11 +3,13 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="19180" windowHeight="7030" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="19180" windowHeight="7030" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="sh1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="sh2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="sh3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="sh31" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +32,14 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -39,7 +49,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -62,13 +72,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1363,4 +1400,3476 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G71"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="26.36328125" customWidth="1" min="1" max="1"/>
+    <col width="38.81640625" customWidth="1" min="2" max="2"/>
+    <col width="18.26953125" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>math</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>chemistry</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ryan Gallagher</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>34</v>
+      </c>
+      <c r="E2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F2" t="n">
+        <v>13</v>
+      </c>
+      <c r="G2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Matthew Kramer</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bhutan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Johnsonfurt</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>45</v>
+      </c>
+      <c r="E3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Jeremy Griffith</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>West Anthonytown</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>16</v>
+      </c>
+      <c r="G4" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Stanley Parks</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Swansonhaven</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>32</v>
+      </c>
+      <c r="E5" t="n">
+        <v>19</v>
+      </c>
+      <c r="F5" t="n">
+        <v>13</v>
+      </c>
+      <c r="G5" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Haley Rhodes</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Farleytown</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>44</v>
+      </c>
+      <c r="E6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" t="n">
+        <v>20</v>
+      </c>
+      <c r="G6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ariel Soto</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Davidmouth</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E7" t="n">
+        <v>13</v>
+      </c>
+      <c r="G7" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Meagan Turner</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Namibia</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>49</v>
+      </c>
+      <c r="F8" t="n">
+        <v>19</v>
+      </c>
+      <c r="G8" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Samuel Castillo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Samoa</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Perryburgh</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>41</v>
+      </c>
+      <c r="F9" t="n">
+        <v>14</v>
+      </c>
+      <c r="G9" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nancy Miller</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>50</v>
+      </c>
+      <c r="E10" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" t="n">
+        <v>18</v>
+      </c>
+      <c r="G10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Jennifer Burns</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Antarctica (the territory South of 60 deg S)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Williamsshire</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>55</v>
+      </c>
+      <c r="E11" t="n">
+        <v>13</v>
+      </c>
+      <c r="F11" t="n">
+        <v>16</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Darrell Smith</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cook Islands</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>South Willie</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>54</v>
+      </c>
+      <c r="F12" t="n">
+        <v>11</v>
+      </c>
+      <c r="G12" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mary Lynch</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Saint Lucia</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>18</v>
+      </c>
+      <c r="E13" t="n">
+        <v>13</v>
+      </c>
+      <c r="G13" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Tina Mays</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>New Kimberly</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>31</v>
+      </c>
+      <c r="E14" t="n">
+        <v>13</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Mr. Julian Everett</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Isle of Man</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>49</v>
+      </c>
+      <c r="E15" t="n">
+        <v>20</v>
+      </c>
+      <c r="G15" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Aaron Fernandez</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Solomon Islands</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Stephentown</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>32</v>
+      </c>
+      <c r="E16" t="n">
+        <v>17</v>
+      </c>
+      <c r="F16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Shannon Lindsey</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>South Georgia and the South Sandwich Islands</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Antonioland</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>23</v>
+      </c>
+      <c r="E17" t="n">
+        <v>20</v>
+      </c>
+      <c r="F17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G17" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Perry Wright</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bouvet Island (Bouvetoya)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>West Kelly</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>28</v>
+      </c>
+      <c r="F18" t="n">
+        <v>8</v>
+      </c>
+      <c r="G18" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Carol Nelson</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Rwanda</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>36</v>
+      </c>
+      <c r="E19" t="n">
+        <v>14</v>
+      </c>
+      <c r="F19" t="n">
+        <v>17</v>
+      </c>
+      <c r="G19" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Brian Collins MD</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>West Daniel</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>50</v>
+      </c>
+      <c r="E20" t="n">
+        <v>10</v>
+      </c>
+      <c r="F20" t="n">
+        <v>15</v>
+      </c>
+      <c r="G20" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Alisha Smith</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cameroon</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Lake Susanmouth</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>50</v>
+      </c>
+      <c r="E21" t="n">
+        <v>17</v>
+      </c>
+      <c r="F21" t="n">
+        <v>12</v>
+      </c>
+      <c r="G21" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Vanessa Mccoy</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Walkertown</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>43</v>
+      </c>
+      <c r="E22" t="n">
+        <v>17</v>
+      </c>
+      <c r="G22" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Mary Simmons</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Saint Pierre and Miquelon</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>37</v>
+      </c>
+      <c r="E23" t="n">
+        <v>9</v>
+      </c>
+      <c r="F23" t="n">
+        <v>9</v>
+      </c>
+      <c r="G23" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Scott Collins</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Wallis and Futuna</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Juliachester</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>54</v>
+      </c>
+      <c r="E24" t="n">
+        <v>11</v>
+      </c>
+      <c r="G24" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Shawn Johnson</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Svalbard &amp; Jan Mayen Islands</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>New Steven</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>57</v>
+      </c>
+      <c r="E25" t="n">
+        <v>15</v>
+      </c>
+      <c r="F25" t="n">
+        <v>6</v>
+      </c>
+      <c r="G25" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Brett Berry</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ukraine</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>45</v>
+      </c>
+      <c r="E26" t="n">
+        <v>16</v>
+      </c>
+      <c r="G26" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Lithuania</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Lake Peterhaven</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>49</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7</v>
+      </c>
+      <c r="G27" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Jennifer Campbell</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>East Meredith</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>54</v>
+      </c>
+      <c r="G28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Jeffrey Adams</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Bhutan</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Randolphstad</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>52</v>
+      </c>
+      <c r="E29" t="n">
+        <v>14</v>
+      </c>
+      <c r="F29" t="n">
+        <v>18</v>
+      </c>
+      <c r="G29" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Nicholas Miller</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>New Jason</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>39</v>
+      </c>
+      <c r="E30" t="n">
+        <v>16</v>
+      </c>
+      <c r="G30" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Isabel Peterson</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>French Guiana</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Port Sherry</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>19</v>
+      </c>
+      <c r="F31" t="n">
+        <v>17</v>
+      </c>
+      <c r="G31" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Juan Garcia</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>20</v>
+      </c>
+      <c r="F32" t="n">
+        <v>12</v>
+      </c>
+      <c r="G32" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>27</v>
+      </c>
+      <c r="E33" t="n">
+        <v>20</v>
+      </c>
+      <c r="G33" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Luis Casey</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Honduras</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>22</v>
+      </c>
+      <c r="E34" t="n">
+        <v>16</v>
+      </c>
+      <c r="F34" t="n">
+        <v>14</v>
+      </c>
+      <c r="G34" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Tiffany Diaz</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>36</v>
+      </c>
+      <c r="E35" t="n">
+        <v>16</v>
+      </c>
+      <c r="F35" t="n">
+        <v>14</v>
+      </c>
+      <c r="G35" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Donald Buchanan</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>36</v>
+      </c>
+      <c r="E36" t="n">
+        <v>7</v>
+      </c>
+      <c r="F36" t="n">
+        <v>15</v>
+      </c>
+      <c r="G36" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Jason Mckenzie</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Somalia</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>East Johnshire</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>44</v>
+      </c>
+      <c r="E37" t="n">
+        <v>9</v>
+      </c>
+      <c r="G37" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Korea</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Lake John</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>24</v>
+      </c>
+      <c r="F38" t="n">
+        <v>12</v>
+      </c>
+      <c r="G38" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Kimberly Cardenas</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>34</v>
+      </c>
+      <c r="E39" t="n">
+        <v>18</v>
+      </c>
+      <c r="G39" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Daniel Stewart</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Anguilla</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Port Toniport</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>56</v>
+      </c>
+      <c r="E40" t="n">
+        <v>12</v>
+      </c>
+      <c r="G40" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Edwardsland</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>22</v>
+      </c>
+      <c r="E41" t="n">
+        <v>12</v>
+      </c>
+      <c r="F41" t="n">
+        <v>15</v>
+      </c>
+      <c r="G41" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Daniel Williamson</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>52</v>
+      </c>
+      <c r="E42" t="n">
+        <v>20</v>
+      </c>
+      <c r="F42" t="n">
+        <v>17</v>
+      </c>
+      <c r="G42" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Deanna Weaver</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>11</v>
+      </c>
+      <c r="F43" t="n">
+        <v>9</v>
+      </c>
+      <c r="G43" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Guyana</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Port Juanmouth</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>23</v>
+      </c>
+      <c r="E44" t="n">
+        <v>17</v>
+      </c>
+      <c r="F44" t="n">
+        <v>15</v>
+      </c>
+      <c r="G44" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Darren Levy</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Armenia</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Jacobshire</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>11</v>
+      </c>
+      <c r="F45" t="n">
+        <v>9</v>
+      </c>
+      <c r="G45" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Bolivia</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>East Jeffreybury</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>43</v>
+      </c>
+      <c r="E46" t="n">
+        <v>8</v>
+      </c>
+      <c r="G46" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Andrea Jones</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>North Macedonia</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>West Karenstad</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>49</v>
+      </c>
+      <c r="E47" t="n">
+        <v>14</v>
+      </c>
+      <c r="F47" t="n">
+        <v>19</v>
+      </c>
+      <c r="G47" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Richard Murphy</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Malawi</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>East Kimberly</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>27</v>
+      </c>
+      <c r="E48" t="n">
+        <v>20</v>
+      </c>
+      <c r="F48" t="n">
+        <v>19</v>
+      </c>
+      <c r="G48" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Michael Davenport</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>36</v>
+      </c>
+      <c r="E49" t="n">
+        <v>9</v>
+      </c>
+      <c r="F49" t="n">
+        <v>20</v>
+      </c>
+      <c r="G49" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Cambodia</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>14</v>
+      </c>
+      <c r="G50" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Eugene Leach</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>East Kerry</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>52</v>
+      </c>
+      <c r="E51" t="n">
+        <v>9</v>
+      </c>
+      <c r="G51" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Mary King</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>7</v>
+      </c>
+      <c r="G52" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Rhonda Dunn</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Mauritius</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Yorkmouth</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>18</v>
+      </c>
+      <c r="E53" t="n">
+        <v>13</v>
+      </c>
+      <c r="F53" t="n">
+        <v>19</v>
+      </c>
+      <c r="G53" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>West Todd</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>59</v>
+      </c>
+      <c r="F54" t="n">
+        <v>20</v>
+      </c>
+      <c r="G54" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Alicia Holt</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Mozambique</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>New David</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>34</v>
+      </c>
+      <c r="E55" t="n">
+        <v>20</v>
+      </c>
+      <c r="F55" t="n">
+        <v>10</v>
+      </c>
+      <c r="G55" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Carolyn Davis</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Libyan Arab Jamahiriya</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>East Allisonhaven</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>59</v>
+      </c>
+      <c r="F56" t="n">
+        <v>20</v>
+      </c>
+      <c r="G56" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Margaret Perez</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Mcdanielbury</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>44</v>
+      </c>
+      <c r="E57" t="n">
+        <v>12</v>
+      </c>
+      <c r="F57" t="n">
+        <v>14</v>
+      </c>
+      <c r="G57" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Tabitha Hill</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Oman</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>North Sandra</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>50</v>
+      </c>
+      <c r="E58" t="n">
+        <v>17</v>
+      </c>
+      <c r="F58" t="n">
+        <v>20</v>
+      </c>
+      <c r="G58" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Ralph Ware</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>37</v>
+      </c>
+      <c r="E59" t="n">
+        <v>11</v>
+      </c>
+      <c r="F59" t="n">
+        <v>17</v>
+      </c>
+      <c r="G59" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Jacqueline Haynes</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Wheelerville</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>56</v>
+      </c>
+      <c r="F60" t="n">
+        <v>14</v>
+      </c>
+      <c r="G60" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Christopher Simmons</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Western Sahara</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>54</v>
+      </c>
+      <c r="E61" t="n">
+        <v>18</v>
+      </c>
+      <c r="G61" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>South Erinstad</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>42</v>
+      </c>
+      <c r="E62" t="n">
+        <v>15</v>
+      </c>
+      <c r="F62" t="n">
+        <v>19</v>
+      </c>
+      <c r="G62" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Wendy Warren</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>34</v>
+      </c>
+      <c r="E63" t="n">
+        <v>17</v>
+      </c>
+      <c r="F63" t="n">
+        <v>7</v>
+      </c>
+      <c r="G63" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Angela Proctor</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>57</v>
+      </c>
+      <c r="E64" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Melissa Miller</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>33</v>
+      </c>
+      <c r="E65" t="n">
+        <v>20</v>
+      </c>
+      <c r="F65" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Wallis and Futuna</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>45</v>
+      </c>
+      <c r="E66" t="n">
+        <v>13</v>
+      </c>
+      <c r="F66" t="n">
+        <v>8</v>
+      </c>
+      <c r="G66" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Martinezfort</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>31</v>
+      </c>
+      <c r="E67" t="n">
+        <v>8</v>
+      </c>
+      <c r="F67" t="n">
+        <v>12</v>
+      </c>
+      <c r="G67" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Susan Guerrero</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Fiji</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>South Kara</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>18</v>
+      </c>
+      <c r="E68" t="n">
+        <v>10</v>
+      </c>
+      <c r="F68" t="n">
+        <v>14</v>
+      </c>
+      <c r="G68" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Amanda Dudley</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Port Jorge</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>29</v>
+      </c>
+      <c r="E69" t="n">
+        <v>11</v>
+      </c>
+      <c r="F69" t="n">
+        <v>8</v>
+      </c>
+      <c r="G69" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Eric Todd</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Syrian Arab Republic</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>46</v>
+      </c>
+      <c r="F70" t="n">
+        <v>18</v>
+      </c>
+      <c r="G70" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Carol Kelly</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Port Jasonfurt</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>31</v>
+      </c>
+      <c r="E71" t="n">
+        <v>11</v>
+      </c>
+      <c r="F71" t="n">
+        <v>18</v>
+      </c>
+      <c r="G71" t="n">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G71"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>math</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>chemistry</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ryan Gallagher</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>34</v>
+      </c>
+      <c r="E2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F2" t="n">
+        <v>13</v>
+      </c>
+      <c r="G2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Matthew Kramer</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bhutan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Johnsonfurt</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>45</v>
+      </c>
+      <c r="E3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Jeremy Griffith</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>West Anthonytown</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>16</v>
+      </c>
+      <c r="G4" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Stanley Parks</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Swansonhaven</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>32</v>
+      </c>
+      <c r="E5" t="n">
+        <v>19</v>
+      </c>
+      <c r="F5" t="n">
+        <v>13</v>
+      </c>
+      <c r="G5" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Haley Rhodes</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Farleytown</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>44</v>
+      </c>
+      <c r="E6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" t="n">
+        <v>20</v>
+      </c>
+      <c r="G6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ariel Soto</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Davidmouth</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E7" t="n">
+        <v>13</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Meagan Turner</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Namibia</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>49</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>19</v>
+      </c>
+      <c r="G8" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Samuel Castillo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Samoa</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Perryburgh</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>41</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="n">
+        <v>14</v>
+      </c>
+      <c r="G9" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nancy Miller</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>50</v>
+      </c>
+      <c r="E10" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" t="n">
+        <v>18</v>
+      </c>
+      <c r="G10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Jennifer Burns</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Antarctica (the territory South of 60 deg S)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Williamsshire</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>55</v>
+      </c>
+      <c r="E11" t="n">
+        <v>13</v>
+      </c>
+      <c r="F11" t="n">
+        <v>16</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Darrell Smith</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cook Islands</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>South Willie</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>54</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="n">
+        <v>11</v>
+      </c>
+      <c r="G12" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mary Lynch</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Saint Lucia</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>18</v>
+      </c>
+      <c r="E13" t="n">
+        <v>13</v>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Tina Mays</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>New Kimberly</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>31</v>
+      </c>
+      <c r="E14" t="n">
+        <v>13</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Mr. Julian Everett</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Isle of Man</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>49</v>
+      </c>
+      <c r="E15" t="n">
+        <v>20</v>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Aaron Fernandez</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Solomon Islands</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Stephentown</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>32</v>
+      </c>
+      <c r="E16" t="n">
+        <v>17</v>
+      </c>
+      <c r="F16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Shannon Lindsey</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>South Georgia and the South Sandwich Islands</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Antonioland</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>23</v>
+      </c>
+      <c r="E17" t="n">
+        <v>20</v>
+      </c>
+      <c r="F17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G17" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Perry Wright</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bouvet Island (Bouvetoya)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>West Kelly</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>28</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="n">
+        <v>8</v>
+      </c>
+      <c r="G18" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Carol Nelson</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Rwanda</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="n">
+        <v>36</v>
+      </c>
+      <c r="E19" t="n">
+        <v>14</v>
+      </c>
+      <c r="F19" t="n">
+        <v>17</v>
+      </c>
+      <c r="G19" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Brian Collins MD</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>West Daniel</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>50</v>
+      </c>
+      <c r="E20" t="n">
+        <v>10</v>
+      </c>
+      <c r="F20" t="n">
+        <v>15</v>
+      </c>
+      <c r="G20" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Alisha Smith</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cameroon</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Lake Susanmouth</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>50</v>
+      </c>
+      <c r="E21" t="n">
+        <v>17</v>
+      </c>
+      <c r="F21" t="n">
+        <v>12</v>
+      </c>
+      <c r="G21" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Vanessa Mccoy</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Walkertown</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>43</v>
+      </c>
+      <c r="E22" t="n">
+        <v>17</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Mary Simmons</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Saint Pierre and Miquelon</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="n">
+        <v>37</v>
+      </c>
+      <c r="E23" t="n">
+        <v>9</v>
+      </c>
+      <c r="F23" t="n">
+        <v>9</v>
+      </c>
+      <c r="G23" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Scott Collins</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Wallis and Futuna</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Juliachester</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>54</v>
+      </c>
+      <c r="E24" t="n">
+        <v>11</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Shawn Johnson</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Svalbard &amp; Jan Mayen Islands</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>New Steven</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>57</v>
+      </c>
+      <c r="E25" t="n">
+        <v>15</v>
+      </c>
+      <c r="F25" t="n">
+        <v>6</v>
+      </c>
+      <c r="G25" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Brett Berry</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ukraine</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="n">
+        <v>45</v>
+      </c>
+      <c r="E26" t="n">
+        <v>16</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Lithuania</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Lake Peterhaven</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>49</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Jennifer Campbell</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>East Meredith</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>54</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Jeffrey Adams</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Bhutan</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Randolphstad</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>52</v>
+      </c>
+      <c r="E29" t="n">
+        <v>14</v>
+      </c>
+      <c r="F29" t="n">
+        <v>18</v>
+      </c>
+      <c r="G29" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Nicholas Miller</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>New Jason</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>39</v>
+      </c>
+      <c r="E30" t="n">
+        <v>16</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Isabel Peterson</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>French Guiana</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Port Sherry</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>19</v>
+      </c>
+      <c r="F31" t="n">
+        <v>17</v>
+      </c>
+      <c r="G31" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Juan Garcia</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="n">
+        <v>20</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="n">
+        <v>12</v>
+      </c>
+      <c r="G32" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>27</v>
+      </c>
+      <c r="E33" t="n">
+        <v>20</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Luis Casey</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Honduras</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>22</v>
+      </c>
+      <c r="E34" t="n">
+        <v>16</v>
+      </c>
+      <c r="F34" t="n">
+        <v>14</v>
+      </c>
+      <c r="G34" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Tiffany Diaz</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="n">
+        <v>36</v>
+      </c>
+      <c r="E35" t="n">
+        <v>16</v>
+      </c>
+      <c r="F35" t="n">
+        <v>14</v>
+      </c>
+      <c r="G35" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Donald Buchanan</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="n">
+        <v>36</v>
+      </c>
+      <c r="E36" t="n">
+        <v>7</v>
+      </c>
+      <c r="F36" t="n">
+        <v>15</v>
+      </c>
+      <c r="G36" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Jason Mckenzie</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Somalia</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>East Johnshire</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>44</v>
+      </c>
+      <c r="E37" t="n">
+        <v>9</v>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Korea</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Lake John</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>24</v>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="n">
+        <v>12</v>
+      </c>
+      <c r="G38" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Kimberly Cardenas</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="n">
+        <v>34</v>
+      </c>
+      <c r="E39" t="n">
+        <v>18</v>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Daniel Stewart</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Anguilla</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Port Toniport</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>56</v>
+      </c>
+      <c r="E40" t="n">
+        <v>12</v>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Edwardsland</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>22</v>
+      </c>
+      <c r="E41" t="n">
+        <v>12</v>
+      </c>
+      <c r="F41" t="n">
+        <v>15</v>
+      </c>
+      <c r="G41" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Daniel Williamson</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="n">
+        <v>52</v>
+      </c>
+      <c r="E42" t="n">
+        <v>20</v>
+      </c>
+      <c r="F42" t="n">
+        <v>17</v>
+      </c>
+      <c r="G42" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Deanna Weaver</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="n">
+        <v>11</v>
+      </c>
+      <c r="F43" t="n">
+        <v>9</v>
+      </c>
+      <c r="G43" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Guyana</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Port Juanmouth</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>23</v>
+      </c>
+      <c r="E44" t="n">
+        <v>17</v>
+      </c>
+      <c r="F44" t="n">
+        <v>15</v>
+      </c>
+      <c r="G44" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Darren Levy</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Armenia</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Jacobshire</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="n">
+        <v>11</v>
+      </c>
+      <c r="F45" t="n">
+        <v>9</v>
+      </c>
+      <c r="G45" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Bolivia</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>East Jeffreybury</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>43</v>
+      </c>
+      <c r="E46" t="n">
+        <v>8</v>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Andrea Jones</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>North Macedonia</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>West Karenstad</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>49</v>
+      </c>
+      <c r="E47" t="n">
+        <v>14</v>
+      </c>
+      <c r="F47" t="n">
+        <v>19</v>
+      </c>
+      <c r="G47" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Richard Murphy</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Malawi</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>East Kimberly</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>27</v>
+      </c>
+      <c r="E48" t="n">
+        <v>20</v>
+      </c>
+      <c r="F48" t="n">
+        <v>19</v>
+      </c>
+      <c r="G48" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Michael Davenport</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>36</v>
+      </c>
+      <c r="E49" t="n">
+        <v>9</v>
+      </c>
+      <c r="F49" t="n">
+        <v>20</v>
+      </c>
+      <c r="G49" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Cambodia</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="n">
+        <v>14</v>
+      </c>
+      <c r="G50" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Eugene Leach</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>East Kerry</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>52</v>
+      </c>
+      <c r="E51" t="n">
+        <v>9</v>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Mary King</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="n">
+        <v>7</v>
+      </c>
+      <c r="G52" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Rhonda Dunn</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Mauritius</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Yorkmouth</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>18</v>
+      </c>
+      <c r="E53" t="n">
+        <v>13</v>
+      </c>
+      <c r="F53" t="n">
+        <v>19</v>
+      </c>
+      <c r="G53" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>West Todd</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>59</v>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="n">
+        <v>20</v>
+      </c>
+      <c r="G54" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Alicia Holt</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Mozambique</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>New David</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>34</v>
+      </c>
+      <c r="E55" t="n">
+        <v>20</v>
+      </c>
+      <c r="F55" t="n">
+        <v>10</v>
+      </c>
+      <c r="G55" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Carolyn Davis</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Libyan Arab Jamahiriya</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>East Allisonhaven</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>59</v>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="n">
+        <v>20</v>
+      </c>
+      <c r="G56" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Margaret Perez</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Mcdanielbury</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>44</v>
+      </c>
+      <c r="E57" t="n">
+        <v>12</v>
+      </c>
+      <c r="F57" t="n">
+        <v>14</v>
+      </c>
+      <c r="G57" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Tabitha Hill</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Oman</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>North Sandra</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>50</v>
+      </c>
+      <c r="E58" t="n">
+        <v>17</v>
+      </c>
+      <c r="F58" t="n">
+        <v>20</v>
+      </c>
+      <c r="G58" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Ralph Ware</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="n">
+        <v>37</v>
+      </c>
+      <c r="E59" t="n">
+        <v>11</v>
+      </c>
+      <c r="F59" t="n">
+        <v>17</v>
+      </c>
+      <c r="G59" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Jacqueline Haynes</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Wheelerville</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>56</v>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="n">
+        <v>14</v>
+      </c>
+      <c r="G60" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Christopher Simmons</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Western Sahara</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="n">
+        <v>54</v>
+      </c>
+      <c r="E61" t="n">
+        <v>18</v>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>South Erinstad</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>42</v>
+      </c>
+      <c r="E62" t="n">
+        <v>15</v>
+      </c>
+      <c r="F62" t="n">
+        <v>19</v>
+      </c>
+      <c r="G62" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Wendy Warren</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="n">
+        <v>34</v>
+      </c>
+      <c r="E63" t="n">
+        <v>17</v>
+      </c>
+      <c r="F63" t="n">
+        <v>7</v>
+      </c>
+      <c r="G63" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Angela Proctor</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="n">
+        <v>57</v>
+      </c>
+      <c r="E64" t="n">
+        <v>20</v>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Melissa Miller</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="n">
+        <v>33</v>
+      </c>
+      <c r="E65" t="n">
+        <v>20</v>
+      </c>
+      <c r="F65" t="n">
+        <v>12</v>
+      </c>
+      <c r="G65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Wallis and Futuna</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="n">
+        <v>45</v>
+      </c>
+      <c r="E66" t="n">
+        <v>13</v>
+      </c>
+      <c r="F66" t="n">
+        <v>8</v>
+      </c>
+      <c r="G66" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Martinezfort</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>31</v>
+      </c>
+      <c r="E67" t="n">
+        <v>8</v>
+      </c>
+      <c r="F67" t="n">
+        <v>12</v>
+      </c>
+      <c r="G67" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Susan Guerrero</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Fiji</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>South Kara</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>18</v>
+      </c>
+      <c r="E68" t="n">
+        <v>10</v>
+      </c>
+      <c r="F68" t="n">
+        <v>14</v>
+      </c>
+      <c r="G68" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Amanda Dudley</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Port Jorge</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>29</v>
+      </c>
+      <c r="E69" t="n">
+        <v>11</v>
+      </c>
+      <c r="F69" t="n">
+        <v>8</v>
+      </c>
+      <c r="G69" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Eric Todd</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Syrian Arab Republic</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="n">
+        <v>46</v>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="n">
+        <v>18</v>
+      </c>
+      <c r="G70" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Carol Kelly</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Port Jasonfurt</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>31</v>
+      </c>
+      <c r="E71" t="n">
+        <v>11</v>
+      </c>
+      <c r="F71" t="n">
+        <v>18</v>
+      </c>
+      <c r="G71" t="n">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>